<commit_message>
migracion inicial a sql
</commit_message>
<xml_diff>
--- a/data/excel/audit_log.xlsx
+++ b/data/excel/audit_log.xlsx
@@ -1703,6 +1703,15 @@
   </x:si>
   <x:si>
     <x:t>0HNMT62TUJQUP:00000001</x:t>
+  </x:si>
+  <x:si>
+    <x:t>6392fc67-6f24-48f1-8cba-3289f099a4b9</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-07-09T13:41:56.5706358Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0HNMTNVBR5UKF:00000001</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -2068,7 +2077,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:S137"/>
+  <x:dimension ref="A1:S138"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="38.139196" style="0" customWidth="1"/>
@@ -7722,6 +7731,44 @@
         <x:v>562</x:v>
       </x:c>
     </x:row>
+    <x:row r="138" spans="1:19">
+      <x:c r="A138" s="0" t="s">
+        <x:v>563</x:v>
+      </x:c>
+      <x:c r="B138" s="0" t="s">
+        <x:v>564</x:v>
+      </x:c>
+      <x:c r="C138" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D138" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E138" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="F138" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="G138" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="I138" s="0" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="L138" s="0" t="s">
+        <x:v>312</x:v>
+      </x:c>
+      <x:c r="M138" s="0" t="s">
+        <x:v>313</x:v>
+      </x:c>
+      <x:c r="O138" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="Q138" s="0" t="s">
+        <x:v>565</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>